<commit_message>
feat(tutors): harden onboarding workflow
Treat signup confirmation as the initial verified session. Retain tutor documents and contracts for admin review, unify roster/card fields, and safely track direct uploads.
</commit_message>
<xml_diff>
--- a/public/seonbae-tutor-card-import-template.xlsx
+++ b/public/seonbae-tutor-card-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="튜터 카드" sheetId="1" r:id="R991df34c66954cea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성 안내" sheetId="2" r:id="R7151218488bf4cb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="튜터 카드" sheetId="1" r:id="R2986ff8f64a94ca8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성 안내" sheetId="2" r:id="Re93e205e031d40d4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -439,7 +439,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>명부 번호</x:v>
+        <x:v>내부 연결 ID</x:v>
       </x:c>
       <x:c r="B1" s="7" t="str">
         <x:v>튜터 이름</x:v>
@@ -448,7 +448,7 @@
         <x:v>시험 / 커리큘럼</x:v>
       </x:c>
       <x:c r="D1" s="7" t="str">
-        <x:v>검증 성적</x:v>
+        <x:v>과목별 성적</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
         <x:v>카테고리</x:v>
@@ -475,7 +475,7 @@
         <x:v>Zoom 호스트 이메일</x:v>
       </x:c>
       <x:c r="M1" s="6" t="str">
-        <x:v>과목별 성적</x:v>
+        <x:v>전공과 학년</x:v>
       </x:c>
       <x:c r="N1" s="6" t="str">
         <x:v>월 가능 시간</x:v>
@@ -3305,13 +3305,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B6" s="26" t="str">
-        <x:v>명부 번호</x:v>
+        <x:v>내부 연결 ID</x:v>
       </x:c>
       <x:c r="C6" s="26" t="str">
-        <x:v>비워 두면 다음 P-xxx 번호가 자동 생성됩니다.</x:v>
+        <x:v>새 카드는 비워 두세요. 저장 시 자동 생성됩니다.</x:v>
       </x:c>
       <x:c r="D6" s="26" t="str">
-        <x:v>기존 번호를 적으면 해당 카드가 수정됩니다.</x:v>
+        <x:v>기존 카드의 내부 ID를 적으면 해당 카드가 수정됩니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
@@ -3373,16 +3373,16 @@
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
       <x:c r="A12" s="12" t="str">
-        <x:v>명부 번호</x:v>
+        <x:v>내부 연결 ID</x:v>
       </x:c>
       <x:c r="B12" s="33" t="str">
         <x:v>선택</x:v>
       </x:c>
       <x:c r="C12" s="12" t="str">
-        <x:v>영문 대문자로 시작, 영문·숫자·하이픈</x:v>
+        <x:v>새 카드는 빈칸. 기존 카드 수정 때만 관리자 화면의 내부 ID 입력</x:v>
       </x:c>
       <x:c r="D12" s="12" t="str">
-        <x:v>P-012 또는 빈칸</x:v>
+        <x:v>T-A1B2C3D4 또는 빈칸</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="38" customHeight="1">
@@ -3415,16 +3415,16 @@
     </x:row>
     <x:row r="15" ht="38" customHeight="1">
       <x:c r="A15" s="12" t="str">
-        <x:v>검증 성적</x:v>
+        <x:v>과목별 성적</x:v>
       </x:c>
       <x:c r="B15" s="33" t="str">
         <x:v>필수</x:v>
       </x:c>
       <x:c r="C15" s="12" t="str">
-        <x:v>카드의 대표 성적</x:v>
+        <x:v>과목:성적을 | 로 구분, 최대 12개</x:v>
       </x:c>
       <x:c r="D15" s="12" t="str">
-        <x:v>43/45</x:v>
+        <x:v>IB Math AA HL:7 | IB Physics HL:7</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="38" customHeight="1">
@@ -3541,16 +3541,16 @@
     </x:row>
     <x:row r="24" ht="38" customHeight="1">
       <x:c r="A24" s="12" t="str">
-        <x:v>과목별 성적</x:v>
+        <x:v>전공과 학년</x:v>
       </x:c>
       <x:c r="B24" s="33" t="str">
         <x:v>선택</x:v>
       </x:c>
       <x:c r="C24" s="12" t="str">
-        <x:v>과목:성적을 | 로 구분, 최대 12개</x:v>
+        <x:v>소개가 비어 있을 때 카드 소개에 반영됩니다.</x:v>
       </x:c>
       <x:c r="D24" s="12" t="str">
-        <x:v>IB Math AA HL:7 | IB Physics HL:7</x:v>
+        <x:v>경제학과 2학년</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="38" customHeight="1">

</xml_diff>